<commit_message>
Integrated Excel download workflow
</commit_message>
<xml_diff>
--- a/outputs/invoice_data.xlsx
+++ b/outputs/invoice_data.xlsx
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>gst</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>total</t>
         </is>
       </c>
     </row>
@@ -441,12 +441,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>520.00</t>
+          <t>4520.00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4520.00</t>
+          <t>Not Found</t>
         </is>
       </c>
     </row>

</xml_diff>